<commit_message>
overpot-barcharts: bar-chart session (components, waterfall BOL/75K, VC Polyol routing)
Recall keyword: overpot-barcharts (see HANDOFF_overpot-barcharts.md).

- Component breakdown grids (Bar_Components_*): 8-bar BOL+75K and 75K-only,
  voltage and current columns; VC Polyol from "Overpotential DATA raw final".
- Waterfall j-V / V-j charts in 4 folders (waterfall/grouped/BOL/75K styles),
  using grid-resolution caches so values match Overpot_grid_* red markers
  (VC Polyol from ALT_DATA). BOL label on top, 75K inside.
- Stacked BOL-vs-75K component grids; 75K-only j-V grid.
- plot_bar_individual_panels.py: KB BM Air BP routed to 260603 repro (0.40 @ 0.7V).
- plot_overpot_dur_300mA_marker.py: Bar_Eta kinetic row y 0.40-0.60.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/260603 New data set (reproducibility)/Overpotential DATA raw alt/Air BP/KB BM/30K/KB BM 1.5bp air_edited.xlsx
+++ b/260603 New data set (reproducibility)/Overpotential DATA raw alt/Air BP/KB BM/30K/KB BM 1.5bp air_edited.xlsx
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="S4" s="0" t="n">
-        <v>-0.5309233673476148</v>
+        <v>-0.492</v>
       </c>
       <c r="V4" s="0" t="n">
         <v>-6</v>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="S5" s="0" t="n">
-        <v>-0.05753919140479981</v>
+        <v>-0.05195</v>
       </c>
       <c r="V5" s="0" t="n">
         <v>-5.9</v>

</xml_diff>